<commit_message>
Change molecular formula to hasDatum Fix celcius units
</commit_message>
<xml_diff>
--- a/test/data/flowcell_excel_schema.xlsx
+++ b/test/data/flowcell_excel_schema.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\battinfoconverter\test\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F2B7665-2652-420A-9F32-19B49CC4E09C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17960783-B62C-4C6A-B325-D9983A7EF352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="24390" windowHeight="20985" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="38700" windowHeight="15345" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="@Schema" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="436">
   <si>
     <t>Metadata</t>
   </si>
@@ -371,9 +371,6 @@
     <t>H2O</t>
   </si>
   <si>
-    <t>hasCatholyte-hasSolvent-hasConstituentA-hasMeasuredProperty-type|molecularFormula-hasStringValue</t>
-  </si>
-  <si>
     <t>Positive electrolyte solvent A purity</t>
   </si>
   <si>
@@ -419,9 +416,6 @@
     <t>Positive electrolyte solvent B chemical formula</t>
   </si>
   <si>
-    <t>hasCatholyte-hasSolvent-hasConstituentB-hasMeasuredProperty-type|molecularFormula-hasStringValue</t>
-  </si>
-  <si>
     <t>Positive electrolyte solvent B purity</t>
   </si>
   <si>
@@ -464,9 +458,6 @@
     <t>K4Fe(CN)6 * 3 H2O</t>
   </si>
   <si>
-    <t>hasCatholyte-hasSolute-hasConstituentA-hasMeasuredProperty-type|molecularFormula-hasStringValue</t>
-  </si>
-  <si>
     <t>Positive electrolyte solute A purity</t>
   </si>
   <si>
@@ -515,9 +506,6 @@
     <t>K3Fe(CN)6</t>
   </si>
   <si>
-    <t>hasCatholyte-hasSolute-hasConstituentB-hasMeasuredProperty-type|molecularFormula-hasStringValue</t>
-  </si>
-  <si>
     <t>Positive electrolyte solute B purity</t>
   </si>
   <si>
@@ -611,9 +599,6 @@
     <t>Positive electrolyte temperature</t>
   </si>
   <si>
-    <t>Â°C</t>
-  </si>
-  <si>
     <t>hasCatholyte-hasMeasuredProperty-CelsiusTemperature</t>
   </si>
   <si>
@@ -671,9 +656,6 @@
     <t>Negative electrolyte solvent A chemical formula</t>
   </si>
   <si>
-    <t>hasAnolyte-hasSolvent-hasConstituentA-hasMeasuredProperty-type|molecularFormula-hasStringValue</t>
-  </si>
-  <si>
     <t>Negative electrolyte solvent A purity</t>
   </si>
   <si>
@@ -710,9 +692,6 @@
     <t>Negative electrolyte solvent B chemical formula</t>
   </si>
   <si>
-    <t>hasAnolyte-hasSolvent-hasConstituentB-hasMeasuredProperty-type|molecularFormula-hasStringValue</t>
-  </si>
-  <si>
     <t>Negative electrolyte solvent B purity</t>
   </si>
   <si>
@@ -755,9 +734,6 @@
     <t>KCrC11H18N2O10</t>
   </si>
   <si>
-    <t>hasAnolyte-hasSolute-hasConstituentA-hasMeasuredProperty-type|molecularFormula-hasStringValue</t>
-  </si>
-  <si>
     <t>Negative electrolyte solute A purity</t>
   </si>
   <si>
@@ -803,9 +779,6 @@
     <t>C11H18N2O8</t>
   </si>
   <si>
-    <t>hasAnolyte-hasSolute-hasConstituentB-hasMeasuredProperty-type|molecularFormula-hasStringValue</t>
-  </si>
-  <si>
     <t>Negative electrolyte solute B purity</t>
   </si>
   <si>
@@ -1335,6 +1308,30 @@
   </si>
   <si>
     <t>PolyetherEtherKetone</t>
+  </si>
+  <si>
+    <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatum-type|molecularFormula-hasStringValue</t>
+  </si>
+  <si>
+    <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatum-type|molecularFormula-hasStringValue</t>
+  </si>
+  <si>
+    <t>hasCatholyte-hasSolute-hasConstituentA-hasDatum-type|molecularFormula-hasStringValue</t>
+  </si>
+  <si>
+    <t>hasCatholyte-hasSolute-hasConstituentB-hasDatum-type|molecularFormula-hasStringValue</t>
+  </si>
+  <si>
+    <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatum-type|molecularFormula-hasStringValue</t>
+  </si>
+  <si>
+    <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatum-type|molecularFormula-hasStringValue</t>
+  </si>
+  <si>
+    <t>hasAnolyte-hasSolute-hasConstituentA-hasDatum-type|molecularFormula-hasStringValue</t>
+  </si>
+  <si>
+    <t>hasAnolyte-hasSolute-hasConstituentB-hasDatum-type|molecularFormula-hasStringValue</t>
   </si>
 </sst>
 </file>
@@ -2136,7 +2133,7 @@
         <v>65</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>425</v>
+        <v>416</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>9</v>
@@ -2145,7 +2142,7 @@
         <v>48</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>426</v>
+        <v>417</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>66</v>
@@ -2235,7 +2232,7 @@
         <v>10</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>426</v>
+        <v>417</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>79</v>
@@ -2400,7 +2397,7 @@
         <v>96</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>425</v>
+        <v>416</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>9</v>
@@ -2409,7 +2406,7 @@
         <v>48</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>66</v>
@@ -2499,7 +2496,7 @@
         <v>10</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="F41" s="11" t="s">
         <v>79</v>
@@ -2581,13 +2578,13 @@
         <v>10</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>115</v>
+        <v>428</v>
       </c>
       <c r="F46" s="14"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B47" s="4">
         <v>100</v>
@@ -2599,16 +2596,16 @@
         <v>19</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F47" s="4"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="B48" s="14" t="s">
         <v>118</v>
-      </c>
-      <c r="B48" s="14" t="s">
-        <v>119</v>
       </c>
       <c r="C48" s="14" t="s">
         <v>9</v>
@@ -2617,15 +2614,15 @@
         <v>19</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>434</v>
+        <v>425</v>
       </c>
       <c r="F48" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B49" s="4">
         <v>100</v>
@@ -2637,13 +2634,13 @@
         <v>10</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F49" s="4"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B50" s="14" t="s">
         <v>27</v>
@@ -2655,16 +2652,16 @@
         <v>19</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F50" s="14"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B51" s="4" t="s">
         <v>125</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>126</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>9</v>
@@ -2673,13 +2670,13 @@
         <v>48</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F51" s="4"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B52" s="14"/>
       <c r="C52" s="14" t="s">
@@ -2689,13 +2686,13 @@
         <v>48</v>
       </c>
       <c r="E52" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F52" s="14"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="4" t="s">
@@ -2705,13 +2702,13 @@
         <v>48</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>131</v>
+        <v>429</v>
       </c>
       <c r="F53" s="4"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B54" s="14"/>
       <c r="C54" s="14" t="s">
@@ -2721,13 +2718,13 @@
         <v>48</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F54" s="14"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="4" t="s">
@@ -2737,15 +2734,15 @@
         <v>48</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B56" s="14">
         <v>0</v>
@@ -2757,13 +2754,13 @@
         <v>10</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F56" s="14"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="4" t="s">
@@ -2773,13 +2770,13 @@
         <v>48</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F57" s="4"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B58" s="14"/>
       <c r="C58" s="14" t="s">
@@ -2789,34 +2786,34 @@
         <v>48</v>
       </c>
       <c r="E58" s="14" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F58" s="14"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E59" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E59" s="4" t="s">
-        <v>143</v>
       </c>
       <c r="F59" s="4"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C60" s="14" t="s">
         <v>9</v>
@@ -2825,13 +2822,13 @@
         <v>10</v>
       </c>
       <c r="E60" s="14" t="s">
-        <v>146</v>
+        <v>430</v>
       </c>
       <c r="F60" s="14"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B61" s="4">
         <v>99</v>
@@ -2843,16 +2840,16 @@
         <v>19</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="F61" s="4"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B62" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C62" s="14" t="s">
         <v>9</v>
@@ -2861,36 +2858,36 @@
         <v>19</v>
       </c>
       <c r="E62" s="14" t="s">
-        <v>428</v>
+        <v>419</v>
       </c>
       <c r="F62" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B63" s="4">
         <v>0.5</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="F63" s="4"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B64" s="14" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C64" s="14" t="s">
         <v>9</v>
@@ -2899,13 +2896,13 @@
         <v>19</v>
       </c>
       <c r="E64" s="14" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F64" s="14"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B65" s="4">
         <v>10504474</v>
@@ -2917,16 +2914,16 @@
         <v>48</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F65" s="4"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B66" s="14" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C66" s="14" t="s">
         <v>9</v>
@@ -2935,16 +2932,16 @@
         <v>48</v>
       </c>
       <c r="E66" s="14" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="F66" s="14"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>9</v>
@@ -2953,13 +2950,13 @@
         <v>48</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>163</v>
+        <v>431</v>
       </c>
       <c r="F67" s="4"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B68" s="14">
         <v>98</v>
@@ -2971,16 +2968,16 @@
         <v>48</v>
       </c>
       <c r="E68" s="14" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="F68" s="14"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>9</v>
@@ -2989,36 +2986,36 @@
         <v>48</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>427</v>
+        <v>418</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="14" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B70" s="14">
         <v>0.1</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D70" s="14" t="s">
         <v>48</v>
       </c>
       <c r="E70" s="14" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="F70" s="14"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>9</v>
@@ -3027,13 +3024,13 @@
         <v>48</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="F71" s="4"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="14" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B72" s="14">
         <v>10266370</v>
@@ -3045,52 +3042,52 @@
         <v>48</v>
       </c>
       <c r="E72" s="14" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F72" s="14"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B73" s="4">
         <v>30</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="F73" s="4"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="14" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B74" s="14">
         <v>60</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D74" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E74" s="14" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="F74" s="14"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>9</v>
@@ -3099,117 +3096,117 @@
         <v>19</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="14" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B76" s="14"/>
       <c r="C76" s="14" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D76" s="14" t="s">
         <v>48</v>
       </c>
       <c r="E76" s="14" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="F76" s="14"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="F77" s="4"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="14" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B78" s="14">
         <v>7.7</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D78" s="14" t="s">
         <v>19</v>
       </c>
       <c r="E78" s="14" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="F78" s="14"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="4" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="4" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F79" s="4"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="14" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B80" s="14">
         <v>23</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>429</v>
+        <v>420</v>
       </c>
       <c r="D80" s="14" t="s">
         <v>19</v>
       </c>
       <c r="E80" s="14" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="F80" s="14"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B81" s="4">
         <v>50</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="F81" s="4"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="14" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B82" s="14"/>
       <c r="C82" s="14" t="s">
@@ -3219,15 +3216,15 @@
         <v>19</v>
       </c>
       <c r="E82" s="14" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="F82" s="14" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="4" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="4" t="s">
@@ -3237,47 +3234,47 @@
         <v>19</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="14" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B84" s="14"/>
       <c r="C84" s="14" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D84" s="14" t="s">
         <v>19</v>
       </c>
       <c r="E84" s="14" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="F84" s="14"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="4" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>48</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="F85" s="4"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -3287,7 +3284,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>27</v>
@@ -3299,13 +3296,13 @@
         <v>10</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="F87" s="4"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B88" s="5"/>
       <c r="C88" s="5" t="s">
@@ -3315,13 +3312,13 @@
         <v>48</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="F88" s="5"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>111</v>
@@ -3333,13 +3330,13 @@
         <v>10</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="F89" s="4"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>114</v>
@@ -3351,13 +3348,13 @@
         <v>10</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>215</v>
+        <v>432</v>
       </c>
       <c r="F90" s="5"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="B91" s="4">
         <v>100</v>
@@ -3369,16 +3366,16 @@
         <v>19</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="F91" s="4"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C92" s="5" t="s">
         <v>9</v>
@@ -3387,15 +3384,15 @@
         <v>19</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>431</v>
+        <v>422</v>
       </c>
       <c r="F92" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B93" s="4">
         <v>100</v>
@@ -3407,13 +3404,13 @@
         <v>10</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="F93" s="4"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>27</v>
@@ -3425,16 +3422,16 @@
         <v>19</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="F94" s="5"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="4" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C95" s="4" t="s">
         <v>9</v>
@@ -3443,13 +3440,13 @@
         <v>48</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="F95" s="4"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="B96" s="5"/>
       <c r="C96" s="5" t="s">
@@ -3459,13 +3456,13 @@
         <v>48</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="F96" s="5"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="4" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="4" t="s">
@@ -3475,13 +3472,13 @@
         <v>48</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>228</v>
+        <v>433</v>
       </c>
       <c r="F97" s="4"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B98" s="5"/>
       <c r="C98" s="5" t="s">
@@ -3491,13 +3488,13 @@
         <v>48</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="F98" s="5"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="4" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="4" t="s">
@@ -3507,15 +3504,15 @@
         <v>48</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B100" s="5">
         <v>0</v>
@@ -3527,13 +3524,13 @@
         <v>10</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="F100" s="5"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="4" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="4" t="s">
@@ -3543,13 +3540,13 @@
         <v>48</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="F101" s="4"/>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="B102" s="5"/>
       <c r="C102" s="5" t="s">
@@ -3559,16 +3556,16 @@
         <v>48</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="F102" s="5"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C103" s="4" t="s">
         <v>9</v>
@@ -3577,16 +3574,16 @@
         <v>10</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="F103" s="4"/>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C104" s="5" t="s">
         <v>9</v>
@@ -3595,13 +3592,13 @@
         <v>10</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>243</v>
+        <v>434</v>
       </c>
       <c r="F104" s="5"/>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="B105" s="4">
         <v>99</v>
@@ -3613,16 +3610,16 @@
         <v>19</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="F105" s="4"/>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C106" s="5" t="s">
         <v>9</v>
@@ -3631,33 +3628,33 @@
         <v>19</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="F106" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="B107" s="4">
         <v>1</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D107" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="F107" s="4"/>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="B108" s="5" t="s">
         <v>27</v>
@@ -3669,13 +3666,13 @@
         <v>19</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="F108" s="5"/>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="4" t="s">
@@ -3685,16 +3682,16 @@
         <v>48</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="F109" s="4"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="C110" s="5" t="s">
         <v>9</v>
@@ -3703,16 +3700,16 @@
         <v>48</v>
       </c>
       <c r="E110" s="5" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="F110" s="5"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="4" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="C111" s="4" t="s">
         <v>9</v>
@@ -3721,13 +3718,13 @@
         <v>48</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>259</v>
+        <v>435</v>
       </c>
       <c r="F111" s="4"/>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="B112" s="5">
         <v>99</v>
@@ -3739,16 +3736,16 @@
         <v>48</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="F112" s="5"/>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="4" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C113" s="4" t="s">
         <v>9</v>
@@ -3757,36 +3754,36 @@
         <v>48</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="B114" s="5">
         <v>0.1</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>48</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="F114" s="5"/>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="C115" s="4" t="s">
         <v>9</v>
@@ -3795,13 +3792,13 @@
         <v>48</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="F115" s="4"/>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="B116" s="5">
         <v>33267</v>
@@ -3813,52 +3810,52 @@
         <v>48</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="F116" s="5"/>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="B117" s="4">
         <v>10</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="F117" s="4"/>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="B118" s="5">
         <v>60</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>10</v>
       </c>
       <c r="E118" s="5" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="F118" s="5"/>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="4" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C119" s="4" t="s">
         <v>9</v>
@@ -3867,120 +3864,120 @@
         <v>19</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>432</v>
+        <v>423</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="5" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="B120" s="5"/>
       <c r="C120" s="5" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>48</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="F120" s="5"/>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="B121" s="4"/>
       <c r="C121" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D121" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="F121" s="4"/>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="B122" s="5">
         <v>8.6999999999999993</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E122" s="5" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="F122" s="5"/>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="4" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="B123" s="4"/>
       <c r="C123" s="4" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D123" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="F123" s="4"/>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="5" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="B124" s="5">
         <v>23</v>
       </c>
       <c r="C124" s="5" t="s">
-        <v>429</v>
+        <v>420</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E124" s="5" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="F124" s="5"/>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="4" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="B125" s="4">
         <v>50</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D125" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="F125" s="4"/>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="5" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="C126" s="5" t="s">
         <v>9</v>
@@ -3989,18 +3986,18 @@
         <v>19</v>
       </c>
       <c r="E126" s="5" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="F126" s="5" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="C127" s="4" t="s">
         <v>9</v>
@@ -4009,47 +4006,47 @@
         <v>19</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="F127" s="4" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="5" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
       <c r="B128" s="5"/>
       <c r="C128" s="5" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D128" s="5" t="s">
         <v>19</v>
       </c>
       <c r="E128" s="5" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="F128" s="5"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" s="4" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="B129" s="4"/>
       <c r="C129" s="4" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D129" s="4" t="s">
         <v>48</v>
       </c>
       <c r="E129" s="4" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="F129" s="4"/>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
@@ -4059,10 +4056,10 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="C131" s="4" t="s">
         <v>9</v>
@@ -4071,18 +4068,18 @@
         <v>10</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" s="5" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="C132" s="5" t="s">
         <v>9</v>
@@ -4091,16 +4088,16 @@
         <v>10</v>
       </c>
       <c r="E132" s="5" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="F132" s="5"/>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" s="4" t="s">
-        <v>304</v>
+        <v>295</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>305</v>
+        <v>296</v>
       </c>
       <c r="C133" s="4" t="s">
         <v>9</v>
@@ -4109,16 +4106,16 @@
         <v>48</v>
       </c>
       <c r="E133" s="4" t="s">
-        <v>306</v>
+        <v>297</v>
       </c>
       <c r="F133" s="4"/>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" s="5" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>436</v>
+        <v>427</v>
       </c>
       <c r="C134" s="5" t="s">
         <v>9</v>
@@ -4127,13 +4124,13 @@
         <v>10</v>
       </c>
       <c r="E134" s="5" t="s">
-        <v>308</v>
+        <v>299</v>
       </c>
       <c r="F134" s="5"/>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" s="4" t="s">
-        <v>309</v>
+        <v>300</v>
       </c>
       <c r="B135" s="4"/>
       <c r="C135" s="4" t="s">
@@ -4143,13 +4140,13 @@
         <v>48</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>310</v>
+        <v>301</v>
       </c>
       <c r="F135" s="4"/>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" s="5" t="s">
-        <v>311</v>
+        <v>302</v>
       </c>
       <c r="B136" s="5">
         <v>30</v>
@@ -4161,29 +4158,29 @@
         <v>19</v>
       </c>
       <c r="E136" s="5" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="F136" s="5"/>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="4" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="B137" s="4"/>
       <c r="C137" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D137" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E137" s="4" t="s">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="F137" s="4"/>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" s="5" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="B138" s="5">
         <v>10</v>
@@ -4195,16 +4192,16 @@
         <v>19</v>
       </c>
       <c r="E138" s="5" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="F138" s="5"/>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="4" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>318</v>
+        <v>309</v>
       </c>
       <c r="C139" s="4" t="s">
         <v>9</v>
@@ -4213,18 +4210,18 @@
         <v>19</v>
       </c>
       <c r="E139" s="4" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="F139" s="4" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" s="5" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="C140" s="5" t="s">
         <v>9</v>
@@ -4233,15 +4230,15 @@
         <v>19</v>
       </c>
       <c r="E140" s="5" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="F140" s="5" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" s="12" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="B141" s="13"/>
       <c r="C141" s="13"/>
@@ -4251,10 +4248,10 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="C142" s="4" t="s">
         <v>9</v>
@@ -4263,16 +4260,16 @@
         <v>10</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>327</v>
+        <v>318</v>
       </c>
       <c r="F142" s="4"/>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" s="14" t="s">
-        <v>328</v>
+        <v>319</v>
       </c>
       <c r="B143" s="14" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
       <c r="C143" s="14" t="s">
         <v>9</v>
@@ -4281,18 +4278,18 @@
         <v>10</v>
       </c>
       <c r="E143" s="14" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
       <c r="F143" s="14" t="s">
-        <v>331</v>
+        <v>322</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
-        <v>332</v>
+        <v>323</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>333</v>
+        <v>324</v>
       </c>
       <c r="C144" s="4" t="s">
         <v>9</v>
@@ -4301,16 +4298,16 @@
         <v>48</v>
       </c>
       <c r="E144" s="4" t="s">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="F144" s="4"/>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" s="14" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="B145" s="14" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="C145" s="14" t="s">
         <v>9</v>
@@ -4319,16 +4316,16 @@
         <v>10</v>
       </c>
       <c r="E145" s="14" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
       <c r="F145" s="14"/>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" s="4" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="C146" s="4" t="s">
         <v>9</v>
@@ -4337,16 +4334,16 @@
         <v>10</v>
       </c>
       <c r="E146" s="4" t="s">
-        <v>433</v>
+        <v>424</v>
       </c>
       <c r="F146" s="4"/>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" s="14" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="B147" s="14" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="C147" s="14" t="s">
         <v>9</v>
@@ -4355,16 +4352,16 @@
         <v>10</v>
       </c>
       <c r="E147" s="14" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="F147" s="14"/>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="C148" s="4" t="s">
         <v>9</v>
@@ -4373,16 +4370,16 @@
         <v>48</v>
       </c>
       <c r="E148" s="4" t="s">
-        <v>345</v>
+        <v>336</v>
       </c>
       <c r="F148" s="4"/>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="14" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="B149" s="14" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="C149" s="14" t="s">
         <v>9</v>
@@ -4391,16 +4388,16 @@
         <v>10</v>
       </c>
       <c r="E149" s="14" t="s">
-        <v>348</v>
+        <v>339</v>
       </c>
       <c r="F149" s="14"/>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
-        <v>349</v>
+        <v>340</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>350</v>
+        <v>341</v>
       </c>
       <c r="C150" s="4" t="s">
         <v>9</v>
@@ -4409,13 +4406,13 @@
         <v>19</v>
       </c>
       <c r="E150" s="4" t="s">
-        <v>351</v>
+        <v>342</v>
       </c>
       <c r="F150" s="4"/>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="14" t="s">
-        <v>352</v>
+        <v>343</v>
       </c>
       <c r="B151" s="14"/>
       <c r="C151" s="14" t="s">
@@ -4425,13 +4422,13 @@
         <v>19</v>
       </c>
       <c r="E151" s="14" t="s">
-        <v>353</v>
+        <v>344</v>
       </c>
       <c r="F151" s="14"/>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" s="4" t="s">
-        <v>354</v>
+        <v>345</v>
       </c>
       <c r="B152" s="4">
         <v>450</v>
@@ -4443,34 +4440,34 @@
         <v>10</v>
       </c>
       <c r="E152" s="4" t="s">
-        <v>355</v>
+        <v>346</v>
       </c>
       <c r="F152" s="4"/>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" s="14" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="B153" s="14">
         <v>6</v>
       </c>
       <c r="C153" s="14" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
       <c r="D153" s="14" t="s">
         <v>19</v>
       </c>
       <c r="E153" s="14" t="s">
-        <v>358</v>
+        <v>349</v>
       </c>
       <c r="F153" s="14"/>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
       <c r="C154" s="4" t="s">
         <v>9</v>
@@ -4479,18 +4476,18 @@
         <v>10</v>
       </c>
       <c r="E154" s="4" t="s">
-        <v>361</v>
+        <v>352</v>
       </c>
       <c r="F154" s="4" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" s="14" t="s">
-        <v>363</v>
+        <v>354</v>
       </c>
       <c r="B155" s="14" t="s">
-        <v>364</v>
+        <v>355</v>
       </c>
       <c r="C155" s="14" t="s">
         <v>9</v>
@@ -4499,10 +4496,10 @@
         <v>19</v>
       </c>
       <c r="E155" s="14" t="s">
-        <v>361</v>
+        <v>352</v>
       </c>
       <c r="F155" s="14" t="s">
-        <v>365</v>
+        <v>356</v>
       </c>
     </row>
   </sheetData>
@@ -4521,66 +4518,66 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>366</v>
+        <v>357</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="B2" t="s">
-        <v>369</v>
+        <v>360</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="B3" t="s">
-        <v>371</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="B4" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>374</v>
+        <v>365</v>
       </c>
       <c r="B5" t="s">
-        <v>375</v>
+        <v>366</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>376</v>
+        <v>367</v>
       </c>
       <c r="B6" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="B7" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="B8" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
     </row>
   </sheetData>
@@ -4600,58 +4597,58 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>366</v>
+        <v>357</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="B2" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="C2" t="s">
-        <v>384</v>
+        <v>375</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>327</v>
+        <v>318</v>
       </c>
       <c r="C3" t="s">
-        <v>385</v>
+        <v>376</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="B4" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="C4" t="s">
-        <v>386</v>
+        <v>377</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>388</v>
+        <v>379</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>389</v>
+        <v>380</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4659,7 +4656,7 @@
         <v>82</v>
       </c>
       <c r="B8" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -4667,47 +4664,47 @@
         <v>44</v>
       </c>
       <c r="B9" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="C10" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
       <c r="B11" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
       <c r="B12" t="s">
-        <v>394</v>
+        <v>385</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>395</v>
+        <v>386</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="B14" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
       <c r="C14" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
     </row>
   </sheetData>
@@ -4727,18 +4724,18 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>366</v>
+        <v>357</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>399</v>
+        <v>390</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>400</v>
+        <v>391</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4748,12 +4745,12 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>401</v>
+        <v>392</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4763,7 +4760,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4771,7 +4768,7 @@
         <v>31</v>
       </c>
       <c r="B8" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -4779,46 +4776,46 @@
         <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>404</v>
+        <v>395</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="B11" t="s">
-        <v>405</v>
+        <v>396</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="B13" t="s">
-        <v>406</v>
+        <v>397</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="B15" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -4831,23 +4828,23 @@
         <v>57</v>
       </c>
       <c r="B17" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="B18" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B19" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -4857,12 +4854,12 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>436</v>
+        <v>427</v>
       </c>
     </row>
   </sheetData>
@@ -4881,10 +4878,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>366</v>
+        <v>357</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -4892,7 +4889,7 @@
         <v>68</v>
       </c>
       <c r="B2" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -4900,47 +4897,47 @@
         <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B4" t="s">
-        <v>414</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B5" t="s">
-        <v>415</v>
+        <v>406</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B6" t="s">
-        <v>416</v>
+        <v>407</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>195</v>
+        <v>420</v>
       </c>
       <c r="B7" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B8" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -4948,39 +4945,39 @@
         <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B10" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B11" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
       <c r="B12" t="s">
-        <v>422</v>
+        <v>413</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B13" t="s">
-        <v>423</v>
+        <v>414</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -4988,7 +4985,7 @@
         <v>75</v>
       </c>
       <c r="B14" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix capitalization, add classes
</commit_message>
<xml_diff>
--- a/test/data/flowcell_excel_schema.xlsx
+++ b/test/data/flowcell_excel_schema.xlsx
@@ -1017,7 +1017,7 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-Substrate-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasPositiveElectrode-Substrate-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-Substrate-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasPositiveElectrode-Substrate-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-Substrate-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasNegativeElectrode-Substrate-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-Substrate-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasNegativeElectrode-Substrate-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F50" s="14" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="E58" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F58" s="14" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="D62" s="14" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>optional</t>
         </is>
       </c>
       <c r="E62" s="14" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolute-hasConstituentA-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasCatholyte-hasSolute-hasConstituentA-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F66" s="14" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolute-hasConstituentA-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasCatholyte-hasSolute-hasConstituentA-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="E74" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolute-hasConstituentB-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasCatholyte-hasSolute-hasConstituentB-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F74" s="14" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolute-hasConstituentB-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasCatholyte-hasSolute-hasConstituentB-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
@@ -3239,7 +3239,7 @@
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F107" s="4" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-hasConstituentA-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasAnolyte-hasSolute-hasConstituentA-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-hasConstituentA-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasAnolyte-hasSolute-hasConstituentA-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F115" s="4" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-hasConstituentB-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasAnolyte-hasSolute-hasConstituentB-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F122" s="5" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-hasConstituentB-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasAnolyte-hasSolute-hasConstituentB-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F123" s="4" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
-          <t>hasSeparator-hasConstituentA-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasSeparator-hasConstituentA-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F147" s="4" t="inlineStr">
@@ -4593,7 +4593,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t>hasSeparator-hasConstituentA-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasSeparator-hasConstituentA-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F148" s="5" t="inlineStr">
@@ -4649,7 +4649,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t>hasSeparator-hasConstituentB-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasSeparator-hasConstituentB-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F150" s="5" t="inlineStr">
@@ -4677,7 +4677,7 @@
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>hasSeparator-hasConstituentB-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasSeparator-hasConstituentB-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F151" s="4" t="inlineStr">
@@ -4981,7 +4981,7 @@
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>hasComponent-FlowField-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasComponent-FlowField-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F162" s="4" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="E163" s="14" t="inlineStr">
         <is>
-          <t>hasComponent-FlowField-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasComponent-FlowField-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F163" s="14" t="inlineStr">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="B167" s="14" t="inlineStr">
         <is>
-          <t>Viton</t>
+          <t>PolymerCompound</t>
         </is>
       </c>
       <c r="C167" s="14" t="inlineStr">
@@ -5144,7 +5144,11 @@
           <t>Gasket material chemical name</t>
         </is>
       </c>
-      <c r="B168" s="4" t="n"/>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>Viton</t>
+        </is>
+      </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
           <t>No Unit</t>
@@ -5157,7 +5161,7 @@
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>hasComponent-Gasket-hasDatum-type|chemicalName-hasStringValue</t>
+          <t>hasComponent-Gasket-hasDatum-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F168" s="4" t="inlineStr">
@@ -5185,7 +5189,7 @@
       </c>
       <c r="E169" s="14" t="inlineStr">
         <is>
-          <t>hasComponent-Gasket-hasDatum-type|chemicalFormula-hasStringValue</t>
+          <t>hasComponent-Gasket-hasDatum-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F169" s="14" t="inlineStr">
@@ -5674,7 +5678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5883,6 +5887,20 @@
       <c r="A22" t="inlineStr">
         <is>
           <t>PolyetherEtherKetone</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PotassiumSaltCompound</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PolymerCompound</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Separate chemical name and formula
</commit_message>
<xml_diff>
--- a/test/data/flowcell_excel_schema.xlsx
+++ b/test/data/flowcell_excel_schema.xlsx
@@ -1017,7 +1017,7 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-Substrate-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasPositiveElectrode-Substrate-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-Substrate-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasPositiveElectrode-Substrate-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Used two 280 µm carbon papers</t>
+          <t>Used two 280 Âµm carbon papers</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-Substrate-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasNegativeElectrode-Substrate-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-Substrate-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasNegativeElectrode-Substrate-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Used two 280 µm carbon papers</t>
+          <t>Used two 280 Âµm carbon papers</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F50" s="14" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="E58" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F58" s="14" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolute-hasConstituentA-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasCatholyte-hasSolute-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F66" s="14" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolute-hasConstituentA-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasCatholyte-hasSolute-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="E74" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolute-hasConstituentB-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasCatholyte-hasSolute-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F74" s="14" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolute-hasConstituentB-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasCatholyte-hasSolute-hasConstituentB-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
@@ -2943,7 +2943,7 @@
       </c>
       <c r="C88" s="14" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>Â°C</t>
         </is>
       </c>
       <c r="D88" s="14" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
@@ -3239,7 +3239,7 @@
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F107" s="4" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-hasConstituentA-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasAnolyte-hasSolute-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-hasConstituentA-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasAnolyte-hasSolute-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F115" s="4" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-hasConstituentB-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasAnolyte-hasSolute-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F122" s="5" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-hasConstituentB-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasAnolyte-hasSolute-hasConstituentB-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F123" s="4" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>Â°C</t>
         </is>
       </c>
       <c r="D136" s="5" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
-          <t>hasSeparator-hasConstituentA-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasSeparator-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F147" s="4" t="inlineStr">
@@ -4593,7 +4593,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t>hasSeparator-hasConstituentA-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasSeparator-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F148" s="5" t="inlineStr">
@@ -4649,7 +4649,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t>hasSeparator-hasConstituentB-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasSeparator-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F150" s="5" t="inlineStr">
@@ -4677,7 +4677,7 @@
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>hasSeparator-hasConstituentB-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasSeparator-hasConstituentB-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F151" s="4" t="inlineStr">
@@ -4981,7 +4981,7 @@
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>hasComponent-FlowField-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasComponent-FlowField-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F162" s="4" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="E163" s="14" t="inlineStr">
         <is>
-          <t>hasComponent-FlowField-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasComponent-FlowField-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F163" s="14" t="inlineStr">
@@ -5161,7 +5161,7 @@
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>hasComponent-Gasket-hasDatum-type|ChemicalName-hasStringValue</t>
+          <t>hasComponent-Gasket-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
       <c r="F168" s="4" t="inlineStr">
@@ -5189,7 +5189,7 @@
       </c>
       <c r="E169" s="14" t="inlineStr">
         <is>
-          <t>hasComponent-Gasket-hasDatum-type|ChemicalFormula-hasStringValue</t>
+          <t>hasComponent-Gasket-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
       <c r="F169" s="14" t="inlineStr">
@@ -5997,7 +5997,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>Â°C</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>

<commit_message>
Fix special characters in template
</commit_message>
<xml_diff>
--- a/test/data/flowcell_excel_schema.xlsx
+++ b/test/data/flowcell_excel_schema.xlsx
@@ -1148,7 +1148,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Used two 280 Âµm carbon papers</t>
+          <t>Used two 280 µm carbon papers</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Used two 280 Âµm carbon papers</t>
+          <t>Used two 280 µm carbon papers</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2943,7 +2943,7 @@
       </c>
       <c r="C88" s="14" t="inlineStr">
         <is>
-          <t>Â°C</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="D88" s="14" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>Â°C</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="D136" s="5" t="inlineStr">
@@ -5997,7 +5997,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Â°C</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>

<commit_message>
Switch flowcell ontology-link, comment col
</commit_message>
<xml_diff>
--- a/test/data/flowcell_excel_schema.xlsx
+++ b/test/data/flowcell_excel_schema.xlsx
@@ -506,8 +506,8 @@
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="160" customWidth="1" min="5" max="5"/>
-    <col width="74" customWidth="1" min="6" max="6"/>
+    <col width="74" customWidth="1" min="5" max="5"/>
+    <col width="160" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -533,12 +533,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Ontology link</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Comment</t>
         </is>
       </c>
     </row>
@@ -577,12 +577,12 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
+          <t>Required, do not change</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
           <t>type|</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Required, do not change</t>
         </is>
       </c>
     </row>
@@ -609,12 +609,12 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
+          <t>Unique ID for cell</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
           <t>schema:productID</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Unique ID for cell</t>
         </is>
       </c>
     </row>
@@ -641,12 +641,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t>Human-friendly name for the cell</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
           <t>schema:name</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Human-friendly name for the cell</t>
         </is>
       </c>
     </row>
@@ -673,12 +673,12 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
+          <t>Assembly date in ISO8601 format (YYYY-MM-DD)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t>schema:dateCreated</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Assembly date in ISO8601 format (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -705,12 +705,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
+          <t>Organisation that made the cell, value should be in @classes with ID</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
           <t>NotOntologize</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Organisation that made the cell, value should be in @classes with ID</t>
         </is>
       </c>
     </row>
@@ -737,12 +737,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t>Person that made the cell, value should be in @classes with ID</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>NotOntologize</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Person that made the cell, value should be in @classes with ID</t>
         </is>
       </c>
     </row>
@@ -767,12 +767,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -797,12 +797,12 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
+          <t>Name of this schema, do not change</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
           <t>Comment</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Name of this schema, do not change</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
+          <t>Version of this schema, do not change</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
           <t>Comment</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Version of this schema, do not change</t>
         </is>
       </c>
     </row>
@@ -871,12 +871,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -899,12 +899,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -923,12 +923,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-schema:productID</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -953,12 +953,12 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
+          <t>CarbonPaper, CarbonFelt, CarbonCloth etc.</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
           <t>hasPositiveElectrode-Substrate</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>CarbonPaper, CarbonFelt, CarbonCloth etc.</t>
         </is>
       </c>
     </row>
@@ -985,12 +985,12 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
           <t>hasPositiveElectrode-Substrate</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -1017,12 +1017,12 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
           <t>hasPositiveElectrode-Substrate-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
           <t>hasPositiveElectrode-Substrate-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-Substrate-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1107,12 +1107,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-Substrate-schema:productID</t>
         </is>
       </c>
-      <c r="F21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -1133,12 +1133,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-Substrate-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1163,12 +1163,12 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
+          <t>Describe stacking of multiple electrode components, leave empty if single elctrode was used</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
           <t>hasPositiveElectrode-Substrate-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Describe stacking of multiple electrode components, leave empty if single elctrode was used</t>
         </is>
       </c>
     </row>
@@ -1191,12 +1191,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-Substrate-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
-      <c r="F24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1217,12 +1217,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-Substrate-hasMeasuredProperty-Area</t>
         </is>
       </c>
-      <c r="F25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -1243,12 +1243,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-Substrate-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1267,12 +1267,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-Substrate-hasMeasuredProperty-Weight</t>
         </is>
       </c>
-      <c r="F27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -1297,12 +1297,12 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
+          <t>Describe treatment conditions (temperature, heat/cool rate, atmosphere, dwell time, etc.)</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
           <t>hasPositiveElectrode-Substrate-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>Describe treatment conditions (temperature, heat/cool rate, atmosphere, dwell time, etc.)</t>
         </is>
       </c>
     </row>
@@ -1339,12 +1339,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode</t>
         </is>
       </c>
-      <c r="F30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
@@ -1367,12 +1367,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1391,12 +1391,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-schema:productID</t>
         </is>
       </c>
-      <c r="F32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
@@ -1421,12 +1421,12 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
+          <t>CarbonPaper, CarbonFelt, CarbonCloth etc.</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
           <t>hasNegativeElectrode-Substrate</t>
-        </is>
-      </c>
-      <c r="F33" s="11" t="inlineStr">
-        <is>
-          <t>CarbonPaper, CarbonFelt, CarbonCloth etc.</t>
         </is>
       </c>
     </row>
@@ -1453,12 +1453,12 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
           <t>hasNegativeElectrode-Substrate</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -1485,12 +1485,12 @@
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
           <t>hasNegativeElectrode-Substrate-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F35" s="11" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -1517,12 +1517,12 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
           <t>hasNegativeElectrode-Substrate-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -1547,12 +1547,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="11" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-Substrate-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -1575,12 +1575,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E38" s="4" t="n"/>
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-Substrate-schema:productID</t>
         </is>
       </c>
-      <c r="F38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
@@ -1601,12 +1601,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-Substrate-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -1631,12 +1631,12 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
+          <t>Describe stacking of multiple electrode components, leave empty if single elctrode was used</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
           <t>hasNegativeElectrode-Substrate-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>Describe stacking of multiple electrode components, leave empty if single elctrode was used</t>
         </is>
       </c>
     </row>
@@ -1659,12 +1659,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="11" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-Substrate-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
-      <c r="F41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -1685,12 +1685,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-Substrate-hasMeasuredProperty-Area</t>
         </is>
       </c>
-      <c r="F42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
@@ -1711,12 +1711,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="11" t="n"/>
+      <c r="F43" s="11" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-Substrate-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -1735,12 +1735,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E44" s="4" t="n"/>
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-Substrate-hasMeasuredProperty-Weight</t>
         </is>
       </c>
-      <c r="F44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
@@ -1765,12 +1765,12 @@
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
+          <t>Describe treatment conditions (temperature, heat/cool rate, atmosphere, dwell time, etc.)</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
           <t>hasNegativeElectrode-Substrate-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F45" s="11" t="inlineStr">
-        <is>
-          <t>Describe treatment conditions (temperature, heat/cool rate, atmosphere, dwell time, etc.)</t>
         </is>
       </c>
     </row>
@@ -1807,12 +1807,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="E47" s="4" t="n"/>
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
@@ -1831,12 +1831,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E48" s="14" t="inlineStr">
+      <c r="E48" s="14" t="n"/>
+      <c r="F48" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-schema:productID</t>
         </is>
       </c>
-      <c r="F48" s="14" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -1861,12 +1861,12 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolvent-hasConstituentA</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -1893,12 +1893,12 @@
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F50" s="14" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F50" s="14" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -1925,12 +1925,12 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolvent-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -1953,12 +1953,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E52" s="14" t="inlineStr">
+      <c r="E52" s="14" t="n"/>
+      <c r="F52" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolvent-hasConstituentA-hasMeasuredProperty-Purity</t>
         </is>
       </c>
-      <c r="F52" s="14" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -1983,12 +1983,12 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
+          <t>State if purity was considered in concentration calculations or not</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolvent-hasConstituentA-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>State if purity was considered in concentration calculations or not</t>
         </is>
       </c>
     </row>
@@ -2011,12 +2011,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E54" s="14" t="inlineStr">
+      <c r="E54" s="14" t="n"/>
+      <c r="F54" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolvent-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
-      <c r="F54" s="14" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -2039,12 +2039,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolvent-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
@@ -2067,12 +2067,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E56" s="14" t="inlineStr">
+      <c r="E56" s="14" t="n"/>
+      <c r="F56" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolvent-hasConstituentA-schema:productID</t>
         </is>
       </c>
-      <c r="F56" s="14" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -2093,12 +2093,12 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolvent-hasConstituentB</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -2121,12 +2121,12 @@
       </c>
       <c r="E58" s="14" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F58" s="14" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F58" s="14" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -2149,12 +2149,12 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolvent-hasConstituentB-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -2175,12 +2175,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E60" s="14" t="inlineStr">
+      <c r="E60" s="14" t="n"/>
+      <c r="F60" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolvent-hasConstituentB-hasMeasuredProperty-Purity</t>
         </is>
       </c>
-      <c r="F60" s="14" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -2201,12 +2201,12 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
+          <t>State if purity was considered in concentration calculations or not</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolvent-hasConstituentB</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>State if purity was considered in concentration calculations or not</t>
         </is>
       </c>
     </row>
@@ -2227,12 +2227,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E62" s="14" t="inlineStr">
+      <c r="E62" s="14" t="n"/>
+      <c r="F62" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolvent-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
-      <c r="F62" s="14" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -2251,12 +2251,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="E63" s="4" t="n"/>
+      <c r="F63" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolvent-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
@@ -2275,12 +2275,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E64" s="14" t="inlineStr">
+      <c r="E64" s="14" t="n"/>
+      <c r="F64" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolvent-hasConstituentB-schema:productID</t>
         </is>
       </c>
-      <c r="F64" s="14" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -2305,12 +2305,12 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolute-hasConstituentA</t>
-        </is>
-      </c>
-      <c r="F65" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -2337,12 +2337,12 @@
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F66" s="14" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolute-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F66" s="14" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -2369,12 +2369,12 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolute-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -2397,12 +2397,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E68" s="14" t="inlineStr">
+      <c r="E68" s="14" t="n"/>
+      <c r="F68" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolute-hasConstituentA-hasMeasuredProperty-Purity</t>
         </is>
       </c>
-      <c r="F68" s="14" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -2427,12 +2427,12 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
+          <t>State if purity was considered in concentration calculations or not</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolute-hasConstituentA-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>State if purity was considered in concentration calculations or not</t>
         </is>
       </c>
     </row>
@@ -2455,12 +2455,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E70" s="14" t="inlineStr">
+      <c r="E70" s="14" t="n"/>
+      <c r="F70" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolute-hasConstituentA-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F70" s="14" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -2483,12 +2483,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E71" s="4" t="inlineStr">
+      <c r="E71" s="4" t="n"/>
+      <c r="F71" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolute-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="14" t="inlineStr">
@@ -2509,12 +2509,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E72" s="14" t="inlineStr">
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolute-hasConstituentA-schema:productID</t>
         </is>
       </c>
-      <c r="F72" s="14" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -2539,12 +2539,12 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolute-hasConstituentB</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -2571,12 +2571,12 @@
       </c>
       <c r="E74" s="14" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F74" s="14" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolute-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F74" s="14" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -2603,12 +2603,12 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolute-hasConstituentB-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -2631,12 +2631,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E76" s="14" t="inlineStr">
+      <c r="E76" s="14" t="n"/>
+      <c r="F76" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolute-hasConstituentB-hasMeasuredProperty-Purity</t>
         </is>
       </c>
-      <c r="F76" s="14" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -2661,12 +2661,12 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
+          <t>State if purity was considered in concentration calculations or not</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasSolute-hasConstituentB-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>State if purity was considered in concentration calculations or not</t>
         </is>
       </c>
     </row>
@@ -2689,12 +2689,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E78" s="14" t="inlineStr">
+      <c r="E78" s="14" t="n"/>
+      <c r="F78" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolute-hasConstituentB-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F78" s="14" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -2717,12 +2717,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E79" s="4" t="inlineStr">
+      <c r="E79" s="4" t="n"/>
+      <c r="F79" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolute-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="14" t="inlineStr">
@@ -2743,12 +2743,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E80" s="14" t="inlineStr">
+      <c r="E80" s="14" t="n"/>
+      <c r="F80" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasSolute-hasConstituentB-schema:productID</t>
         </is>
       </c>
-      <c r="F80" s="14" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -2769,12 +2769,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E81" s="4" t="inlineStr">
+      <c r="E81" s="4" t="n"/>
+      <c r="F81" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte-hasMeasuredProperty-Volume</t>
         </is>
       </c>
-      <c r="F81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="14" t="inlineStr">
@@ -2795,12 +2795,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E82" s="14" t="inlineStr">
+      <c r="E82" s="14" t="n"/>
+      <c r="F82" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasMeasuredProperty-VolumeFlowRate</t>
         </is>
       </c>
-      <c r="F82" s="14" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -2825,12 +2825,12 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
+          <t>Comment if calibrated differently</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasMeasuredProperty-VolumeFlowRate-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>Comment if calibrated differently</t>
         </is>
       </c>
     </row>
@@ -2851,12 +2851,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E84" s="14" t="inlineStr">
+      <c r="E84" s="14" t="n"/>
+      <c r="F84" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasMeasuredProperty-Pressure</t>
         </is>
       </c>
-      <c r="F84" s="14" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -2875,12 +2875,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E85" s="4" t="inlineStr">
+      <c r="E85" s="4" t="n"/>
+      <c r="F85" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte-hasMeasuredProperty-ElectrolyticConductivity</t>
         </is>
       </c>
-      <c r="F85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="14" t="inlineStr">
@@ -2901,12 +2901,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E86" s="14" t="inlineStr">
+      <c r="E86" s="14" t="n"/>
+      <c r="F86" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasMeasuredProperty-pH</t>
         </is>
       </c>
-      <c r="F86" s="14" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -2925,12 +2925,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E87" s="4" t="inlineStr">
+      <c r="E87" s="4" t="n"/>
+      <c r="F87" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte-hasMeasuredProperty-Density</t>
         </is>
       </c>
-      <c r="F87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
@@ -2951,12 +2951,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E88" s="14" t="inlineStr">
+      <c r="E88" s="14" t="n"/>
+      <c r="F88" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte-hasMeasuredProperty-CelsiusTemperature</t>
         </is>
       </c>
-      <c r="F88" s="14" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -2977,12 +2977,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E89" s="4" t="inlineStr">
+      <c r="E89" s="4" t="n"/>
+      <c r="F89" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte-hasComponent-type|AnolyteTank-hasMeasuredProperty-Volume</t>
         </is>
       </c>
-      <c r="F89" s="4" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
@@ -3003,12 +3003,12 @@
       </c>
       <c r="E90" s="14" t="inlineStr">
         <is>
+          <t>Describe mode of mixing, bubble with gas, magnetic stirrer, leave empty if none</t>
+        </is>
+      </c>
+      <c r="F90" s="14" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasComponent-type|AnolyteTank</t>
-        </is>
-      </c>
-      <c r="F90" s="14" t="inlineStr">
-        <is>
-          <t>Describe mode of mixing, bubble with gas, magnetic stirrer, leave empty if none</t>
         </is>
       </c>
     </row>
@@ -3031,12 +3031,12 @@
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
+          <t>Bubbled with Argon, Nitrogen, leave empty if none</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
           <t>hasCatholyte</t>
-        </is>
-      </c>
-      <c r="F91" s="4" t="inlineStr">
-        <is>
-          <t>Bubbled with Argon, Nitrogen, leave empty if none</t>
         </is>
       </c>
     </row>
@@ -3057,12 +3057,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E92" s="14" t="inlineStr">
+      <c r="E92" s="14" t="n"/>
+      <c r="F92" s="14" t="inlineStr">
         <is>
           <t>hasCatholyte</t>
         </is>
       </c>
-      <c r="F92" s="14" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -3081,12 +3081,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E93" s="4" t="inlineStr">
+      <c r="E93" s="4" t="n"/>
+      <c r="F93" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte</t>
         </is>
       </c>
-      <c r="F93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3121,12 +3121,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E95" s="4" t="inlineStr">
+      <c r="E95" s="4" t="n"/>
+      <c r="F95" s="4" t="inlineStr">
         <is>
           <t>hasAnolyte-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
@@ -3145,12 +3145,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E96" s="5" t="inlineStr">
+      <c r="E96" s="5" t="n"/>
+      <c r="F96" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-schema:productID</t>
         </is>
       </c>
-      <c r="F96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -3175,12 +3175,12 @@
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA</t>
-        </is>
-      </c>
-      <c r="F97" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -3207,12 +3207,12 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F98" s="5" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3239,12 @@
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F99" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -3267,12 +3267,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E100" s="5" t="inlineStr">
+      <c r="E100" s="5" t="n"/>
+      <c r="F100" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-hasMeasuredProperty-Purity</t>
         </is>
       </c>
-      <c r="F100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -3297,12 +3297,12 @@
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
+          <t>State if purity was considered in concentration calculations or not</t>
+        </is>
+      </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F101" s="4" t="inlineStr">
-        <is>
-          <t>State if purity was considered in concentration calculations or not</t>
         </is>
       </c>
     </row>
@@ -3325,12 +3325,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E102" s="5" t="inlineStr">
+      <c r="E102" s="5" t="n"/>
+      <c r="F102" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
-      <c r="F102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -3353,12 +3353,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E103" s="4" t="inlineStr">
+      <c r="E103" s="4" t="n"/>
+      <c r="F103" s="4" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
@@ -3381,12 +3381,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E104" s="5" t="inlineStr">
+      <c r="E104" s="5" t="n"/>
+      <c r="F104" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-schema:productID</t>
         </is>
       </c>
-      <c r="F104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -3407,12 +3407,12 @@
       </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB</t>
-        </is>
-      </c>
-      <c r="F105" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -3435,12 +3435,12 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F106" s="5" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -3463,12 +3463,12 @@
       </c>
       <c r="E107" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F107" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F107" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -3489,12 +3489,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E108" s="5" t="inlineStr">
+      <c r="E108" s="5" t="n"/>
+      <c r="F108" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB-hasMeasuredProperty-Purity</t>
         </is>
       </c>
-      <c r="F108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -3515,12 +3515,12 @@
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
+          <t>State if purity was considered in concentration calculations or not</t>
+        </is>
+      </c>
+      <c r="F109" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB</t>
-        </is>
-      </c>
-      <c r="F109" s="4" t="inlineStr">
-        <is>
-          <t>State if purity was considered in concentration calculations or not</t>
         </is>
       </c>
     </row>
@@ -3543,12 +3543,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E110" s="5" t="inlineStr">
+      <c r="E110" s="5" t="n"/>
+      <c r="F110" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
-      <c r="F110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -3567,12 +3567,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E111" s="4" t="inlineStr">
+      <c r="E111" s="4" t="n"/>
+      <c r="F111" s="4" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -3591,12 +3591,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E112" s="5" t="inlineStr">
+      <c r="E112" s="5" t="n"/>
+      <c r="F112" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB-schema:productID</t>
         </is>
       </c>
-      <c r="F112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -3621,12 +3621,12 @@
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F113" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolute-hasConstituentA</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -3653,12 +3653,12 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F114" s="5" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -3685,12 +3685,12 @@
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F115" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F115" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -3713,12 +3713,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E116" s="5" t="inlineStr">
+      <c r="E116" s="5" t="n"/>
+      <c r="F116" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-hasMeasuredProperty-Purity</t>
         </is>
       </c>
-      <c r="F116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -3743,12 +3743,12 @@
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
+          <t>State if purity was considered in concentration calculations or not</t>
+        </is>
+      </c>
+      <c r="F117" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F117" s="4" t="inlineStr">
-        <is>
-          <t>State if purity was considered in concentration calculations or not</t>
         </is>
       </c>
     </row>
@@ -3771,12 +3771,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E118" s="5" t="inlineStr">
+      <c r="E118" s="5" t="n"/>
+      <c r="F118" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -3799,12 +3799,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E119" s="4" t="inlineStr">
+      <c r="E119" s="4" t="n"/>
+      <c r="F119" s="4" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
@@ -3823,12 +3823,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E120" s="5" t="inlineStr">
+      <c r="E120" s="5" t="n"/>
+      <c r="F120" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-schema:productID</t>
         </is>
       </c>
-      <c r="F120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -3849,12 +3849,12 @@
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolute-hasConstituentB</t>
-        </is>
-      </c>
-      <c r="F121" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -3881,12 +3881,12 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F122" s="5" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -3913,12 +3913,12 @@
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F123" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -3941,12 +3941,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E124" s="5" t="inlineStr">
+      <c r="E124" s="5" t="n"/>
+      <c r="F124" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-hasMeasuredProperty-Purity</t>
         </is>
       </c>
-      <c r="F124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -3971,12 +3971,12 @@
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
+          <t>State if purity was considered in concentration calculations or not</t>
+        </is>
+      </c>
+      <c r="F125" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F125" s="4" t="inlineStr">
-        <is>
-          <t>State if purity was considered in concentration calculations or not</t>
         </is>
       </c>
     </row>
@@ -3999,12 +3999,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E126" s="5" t="inlineStr">
+      <c r="E126" s="5" t="n"/>
+      <c r="F126" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -4027,12 +4027,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E127" s="4" t="inlineStr">
+      <c r="E127" s="4" t="n"/>
+      <c r="F127" s="4" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F127" s="4" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
@@ -4053,12 +4053,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E128" s="5" t="inlineStr">
+      <c r="E128" s="5" t="n"/>
+      <c r="F128" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-schema:productID</t>
         </is>
       </c>
-      <c r="F128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -4079,12 +4079,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E129" s="4" t="inlineStr">
+      <c r="E129" s="4" t="n"/>
+      <c r="F129" s="4" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-Volume</t>
         </is>
       </c>
-      <c r="F129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
@@ -4105,12 +4105,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E130" s="5" t="inlineStr">
+      <c r="E130" s="5" t="n"/>
+      <c r="F130" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-VolumeFlowRate</t>
         </is>
       </c>
-      <c r="F130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -4135,12 +4135,12 @@
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
+          <t>Comment if calibrated differently</t>
+        </is>
+      </c>
+      <c r="F131" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-hasMeasuredProperty-VolumeFlowRate-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F131" s="4" t="inlineStr">
-        <is>
-          <t>Comment if calibrated differently</t>
         </is>
       </c>
     </row>
@@ -4161,12 +4161,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E132" s="5" t="inlineStr">
+      <c r="E132" s="5" t="n"/>
+      <c r="F132" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-Pressure</t>
         </is>
       </c>
-      <c r="F132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -4185,12 +4185,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E133" s="4" t="inlineStr">
+      <c r="E133" s="4" t="n"/>
+      <c r="F133" s="4" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-ElectrolyticConductivity</t>
         </is>
       </c>
-      <c r="F133" s="4" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
@@ -4211,12 +4211,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E134" s="5" t="inlineStr">
+      <c r="E134" s="5" t="n"/>
+      <c r="F134" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-pH</t>
         </is>
       </c>
-      <c r="F134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -4235,12 +4235,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E135" s="4" t="inlineStr">
+      <c r="E135" s="4" t="n"/>
+      <c r="F135" s="4" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-Density</t>
         </is>
       </c>
-      <c r="F135" s="4" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
@@ -4261,12 +4261,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E136" s="5" t="inlineStr">
+      <c r="E136" s="5" t="n"/>
+      <c r="F136" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-CelsiusTemperature</t>
         </is>
       </c>
-      <c r="F136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -4287,12 +4287,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E137" s="4" t="inlineStr">
+      <c r="E137" s="4" t="n"/>
+      <c r="F137" s="4" t="inlineStr">
         <is>
           <t>hasCatholyte-hasComponent-type|AnolyteTank-hasMeasuredProperty-Volume</t>
         </is>
       </c>
-      <c r="F137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
@@ -4317,12 +4317,12 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
+          <t>Describe mode of mixing, bubble with gas, magnetic stirrer, leave empty if none</t>
+        </is>
+      </c>
+      <c r="F138" s="5" t="inlineStr">
+        <is>
           <t>hasCatholyte-hasComponent-type|AnolyteTank-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F138" s="5" t="inlineStr">
-        <is>
-          <t>Describe mode of mixing, bubble with gas, magnetic stirrer, leave empty if none</t>
         </is>
       </c>
     </row>
@@ -4349,12 +4349,12 @@
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
+          <t>Bubbled with Argon, Nitrogen, leave empty if none</t>
+        </is>
+      </c>
+      <c r="F139" s="4" t="inlineStr">
+        <is>
           <t>hasAnolyte-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F139" s="4" t="inlineStr">
-        <is>
-          <t>Bubbled with Argon, Nitrogen, leave empty if none</t>
         </is>
       </c>
     </row>
@@ -4375,12 +4375,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E140" s="5" t="inlineStr">
+      <c r="E140" s="5" t="n"/>
+      <c r="F140" s="5" t="inlineStr">
         <is>
           <t>hasAnolyte</t>
         </is>
       </c>
-      <c r="F140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -4399,12 +4399,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E141" s="4" t="inlineStr">
+      <c r="E141" s="4" t="n"/>
+      <c r="F141" s="4" t="inlineStr">
         <is>
           <t>hasAnolyte</t>
         </is>
       </c>
-      <c r="F141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -4441,12 +4441,12 @@
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
+          <t>CationExchangeMembrane, AnionExchangeMembrane</t>
+        </is>
+      </c>
+      <c r="F143" s="4" t="inlineStr">
+        <is>
           <t>hasSeparator</t>
-        </is>
-      </c>
-      <c r="F143" s="4" t="inlineStr">
-        <is>
-          <t>CationExchangeMembrane, AnionExchangeMembrane</t>
         </is>
       </c>
     </row>
@@ -4471,12 +4471,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E144" s="5" t="inlineStr">
+      <c r="E144" s="5" t="n"/>
+      <c r="F144" s="5" t="inlineStr">
         <is>
           <t>hasSeparator-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -4499,12 +4499,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E145" s="4" t="inlineStr">
+      <c r="E145" s="4" t="n"/>
+      <c r="F145" s="4" t="inlineStr">
         <is>
           <t>hasSeparator-schema:productID</t>
         </is>
       </c>
-      <c r="F145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
@@ -4529,12 +4529,12 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
           <t>hasSeparator-hasConstituentA</t>
-        </is>
-      </c>
-      <c r="F146" s="5" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -4561,12 +4561,12 @@
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F147" s="4" t="inlineStr">
+        <is>
           <t>hasSeparator-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F147" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -4593,12 +4593,12 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F148" s="5" t="inlineStr">
+        <is>
           <t>hasSeparator-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F148" s="5" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -4621,12 +4621,12 @@
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F149" s="4" t="inlineStr">
+        <is>
           <t>hasSeparator-hasConstituentB</t>
-        </is>
-      </c>
-      <c r="F149" s="4" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -4649,12 +4649,12 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F150" s="5" t="inlineStr">
+        <is>
           <t>hasSeparator-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F150" s="5" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -4677,12 +4677,12 @@
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F151" s="4" t="inlineStr">
+        <is>
           <t>hasSeparator-hasConstituentB-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F151" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -4705,12 +4705,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E152" s="5" t="inlineStr">
+      <c r="E152" s="5" t="n"/>
+      <c r="F152" s="5" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -4729,12 +4729,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E153" s="4" t="inlineStr">
+      <c r="E153" s="4" t="n"/>
+      <c r="F153" s="4" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-ElectrolyticConductivity</t>
         </is>
       </c>
-      <c r="F153" s="4" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="5" t="inlineStr">
@@ -4755,12 +4755,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E154" s="5" t="inlineStr">
+      <c r="E154" s="5" t="n"/>
+      <c r="F154" s="5" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Area</t>
         </is>
       </c>
-      <c r="F154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -4785,12 +4785,12 @@
       </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
+          <t>Describe membrane storage conditions (medium, duration, temperature)</t>
+        </is>
+      </c>
+      <c r="F155" s="4" t="inlineStr">
+        <is>
           <t>hasSeparator-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F155" s="4" t="inlineStr">
-        <is>
-          <t>Describe membrane storage conditions (medium, duration, temperature)</t>
         </is>
       </c>
     </row>
@@ -4817,12 +4817,12 @@
       </c>
       <c r="E156" s="5" t="inlineStr">
         <is>
+          <t>Describe membrane pre-treatment conditions (medium, duration, temperature)</t>
+        </is>
+      </c>
+      <c r="F156" s="5" t="inlineStr">
+        <is>
           <t>hasSeparator-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F156" s="5" t="inlineStr">
-        <is>
-          <t>Describe membrane pre-treatment conditions (medium, duration, temperature)</t>
         </is>
       </c>
     </row>
@@ -4859,12 +4859,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E158" s="4" t="inlineStr">
+      <c r="E158" s="4" t="n"/>
+      <c r="F158" s="4" t="inlineStr">
         <is>
           <t>hasCase</t>
         </is>
       </c>
-      <c r="F158" s="4" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="14" t="inlineStr">
@@ -4889,12 +4889,12 @@
       </c>
       <c r="E159" s="14" t="inlineStr">
         <is>
+          <t>Fuel Cell Technologies, Pinflow, etc.</t>
+        </is>
+      </c>
+      <c r="F159" s="14" t="inlineStr">
+        <is>
           <t>hasCase-schema:manufacturer</t>
-        </is>
-      </c>
-      <c r="F159" s="14" t="inlineStr">
-        <is>
-          <t>Fuel Cell Technologies, Pinflow, etc.</t>
         </is>
       </c>
     </row>
@@ -4919,12 +4919,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E160" s="4" t="inlineStr">
+      <c r="E160" s="4" t="n"/>
+      <c r="F160" s="4" t="inlineStr">
         <is>
           <t>hasCase-schema:productID</t>
         </is>
       </c>
-      <c r="F160" s="4" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="14" t="inlineStr">
@@ -4949,12 +4949,12 @@
       </c>
       <c r="E161" s="14" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F161" s="14" t="inlineStr">
+        <is>
           <t>hasComponent-FlowField</t>
-        </is>
-      </c>
-      <c r="F161" s="14" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -4981,12 +4981,12 @@
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F162" s="4" t="inlineStr">
+        <is>
           <t>hasComponent-FlowField-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F162" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -5013,12 +5013,12 @@
       </c>
       <c r="E163" s="14" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F163" s="14" t="inlineStr">
+        <is>
           <t>hasComponent-FlowField-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F163" s="14" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -5043,12 +5043,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E164" s="4" t="inlineStr">
+      <c r="E164" s="4" t="n"/>
+      <c r="F164" s="4" t="inlineStr">
         <is>
           <t>hasComponent-FlowField-schema:description</t>
         </is>
       </c>
-      <c r="F164" s="4" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="14" t="inlineStr">
@@ -5071,12 +5071,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E165" s="14" t="inlineStr">
+      <c r="E165" s="14" t="n"/>
+      <c r="F165" s="14" t="inlineStr">
         <is>
           <t>hasComponent-FlowField-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F165" s="14" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
@@ -5099,12 +5099,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E166" s="4" t="inlineStr">
+      <c r="E166" s="4" t="n"/>
+      <c r="F166" s="4" t="inlineStr">
         <is>
           <t>hasComponent-FlowField-schema:productID</t>
         </is>
       </c>
-      <c r="F166" s="4" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="14" t="inlineStr">
@@ -5129,12 +5129,12 @@
       </c>
       <c r="E167" s="14" t="inlineStr">
         <is>
+          <t>Ontology term, be as specific as possible</t>
+        </is>
+      </c>
+      <c r="F167" s="14" t="inlineStr">
+        <is>
           <t>hasComponent-Gasket</t>
-        </is>
-      </c>
-      <c r="F167" s="14" t="inlineStr">
-        <is>
-          <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
     </row>
@@ -5161,12 +5161,12 @@
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F168" s="4" t="inlineStr">
+        <is>
           <t>hasComponent-Gasket-hasDatumA-type|ChemicalName-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F168" s="4" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -5189,12 +5189,12 @@
       </c>
       <c r="E169" s="14" t="inlineStr">
         <is>
+          <t>Important if specific ontology class not available</t>
+        </is>
+      </c>
+      <c r="F169" s="14" t="inlineStr">
+        <is>
           <t>hasComponent-Gasket-hasDatumB-type|ChemicalFormula-hasStringValue</t>
-        </is>
-      </c>
-      <c r="F169" s="14" t="inlineStr">
-        <is>
-          <t>Important if specific ontology class not available</t>
         </is>
       </c>
     </row>
@@ -5219,12 +5219,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E170" s="4" t="inlineStr">
+      <c r="E170" s="4" t="n"/>
+      <c r="F170" s="4" t="inlineStr">
         <is>
           <t>hasComponent-Gasket-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F170" s="4" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="14" t="inlineStr">
@@ -5243,12 +5243,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E171" s="14" t="inlineStr">
+      <c r="E171" s="14" t="n"/>
+      <c r="F171" s="14" t="inlineStr">
         <is>
           <t>hasComponent-Gasket-schema:productID</t>
         </is>
       </c>
-      <c r="F171" s="14" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
@@ -5269,12 +5269,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E172" s="4" t="inlineStr">
+      <c r="E172" s="4" t="n"/>
+      <c r="F172" s="4" t="inlineStr">
         <is>
           <t>hasComponent-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F172" s="4" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="14" t="inlineStr">
@@ -5295,12 +5295,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E173" s="14" t="inlineStr">
+      <c r="E173" s="14" t="n"/>
+      <c r="F173" s="14" t="inlineStr">
         <is>
           <t>hasCase-hasMeasuredProperty-Torque</t>
         </is>
       </c>
-      <c r="F173" s="14" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -5325,12 +5325,12 @@
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
+          <t>Describe cell lead-instrument connection</t>
+        </is>
+      </c>
+      <c r="F174" s="4" t="inlineStr">
+        <is>
           <t>hasComponent-Connector-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F174" s="4" t="inlineStr">
-        <is>
-          <t>Describe cell lead-instrument connection</t>
         </is>
       </c>
     </row>
@@ -5357,12 +5357,12 @@
       </c>
       <c r="E175" s="14" t="inlineStr">
         <is>
+          <t>Describe if other mode, e.g. 2-point</t>
+        </is>
+      </c>
+      <c r="F175" s="14" t="inlineStr">
+        <is>
           <t>hasComponent-Connector-rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F175" s="14" t="inlineStr">
-        <is>
-          <t>Describe if other mode, e.g. 2-point</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update pytest expected vals
</commit_message>
<xml_diff>
--- a/test/data/flowcell_excel_schema.xlsx
+++ b/test/data/flowcell_excel_schema.xlsx
@@ -38,7 +38,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -85,6 +85,26 @@
         <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB1A0C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDA9694"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2DCDB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -98,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -132,6 +152,20 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3141,16 +3175,16 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="inlineStr">
+      <c r="A95" s="15" t="inlineStr">
         <is>
           <t>Negative electrolyte / negolyte / anolyte</t>
         </is>
       </c>
-      <c r="B95" s="3" t="n"/>
-      <c r="C95" s="3" t="n"/>
-      <c r="D95" s="3" t="n"/>
-      <c r="E95" s="3" t="n"/>
-      <c r="F95" s="3" t="n"/>
+      <c r="B95" s="16" t="n"/>
+      <c r="C95" s="16" t="n"/>
+      <c r="D95" s="16" t="n"/>
+      <c r="E95" s="16" t="n"/>
+      <c r="F95" s="16" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -3181,28 +3215,28 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="5" t="inlineStr">
+      <c r="A97" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte manufacturer product ID</t>
         </is>
       </c>
-      <c r="B97" s="5" t="inlineStr">
+      <c r="B97" s="17" t="inlineStr">
         <is>
           <t>Negolyte 1M</t>
         </is>
       </c>
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D97" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E97" s="5" t="n"/>
-      <c r="F97" s="5" t="inlineStr">
+      <c r="C97" s="17" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D97" s="17" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E97" s="17" t="n"/>
+      <c r="F97" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-schema:productID</t>
         </is>
@@ -3241,32 +3275,32 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="inlineStr">
+      <c r="A99" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solvent A chemical name</t>
         </is>
       </c>
-      <c r="B99" s="5" t="inlineStr">
+      <c r="B99" s="17" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="C99" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D99" s="5" t="inlineStr">
+      <c r="C99" s="17" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D99" s="17" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E99" s="5" t="inlineStr">
+      <c r="E99" s="17" t="inlineStr">
         <is>
           <t>Important if specific ontology class not available</t>
         </is>
       </c>
-      <c r="F99" s="5" t="inlineStr">
+      <c r="F99" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
@@ -3305,26 +3339,26 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="inlineStr">
+      <c r="A101" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solvent A purity</t>
         </is>
       </c>
-      <c r="B101" s="5" t="n">
+      <c r="B101" s="17" t="n">
         <v>100</v>
       </c>
-      <c r="C101" s="5" t="inlineStr">
+      <c r="C101" s="17" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D101" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E101" s="5" t="n"/>
-      <c r="F101" s="5" t="inlineStr">
+      <c r="D101" s="17" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E101" s="17" t="n"/>
+      <c r="F101" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-hasMeasuredProperty-Purity</t>
         </is>
@@ -3363,26 +3397,26 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="inlineStr">
+      <c r="A103" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solvent A volume fraction</t>
         </is>
       </c>
-      <c r="B103" s="5" t="n">
+      <c r="B103" s="17" t="n">
         <v>100</v>
       </c>
-      <c r="C103" s="5" t="inlineStr">
+      <c r="C103" s="17" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D103" s="5" t="inlineStr">
+      <c r="D103" s="17" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E103" s="5" t="n"/>
-      <c r="F103" s="5" t="inlineStr">
+      <c r="E103" s="17" t="n"/>
+      <c r="F103" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
         </is>
@@ -3417,28 +3451,28 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="inlineStr">
+      <c r="A105" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solvent A manufacturer product ID</t>
         </is>
       </c>
-      <c r="B105" s="5" t="inlineStr">
+      <c r="B105" s="17" t="inlineStr">
         <is>
           <t>MilliQ</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D105" s="5" t="inlineStr">
+      <c r="C105" s="17" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D105" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E105" s="5" t="n"/>
-      <c r="F105" s="5" t="inlineStr">
+      <c r="E105" s="17" t="n"/>
+      <c r="F105" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentA-schema:productID</t>
         </is>
@@ -3473,28 +3507,28 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="5" t="inlineStr">
+      <c r="A107" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solvent B chemical name</t>
         </is>
       </c>
-      <c r="B107" s="5" t="n"/>
-      <c r="C107" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D107" s="5" t="inlineStr">
+      <c r="B107" s="17" t="n"/>
+      <c r="C107" s="17" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D107" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E107" s="5" t="inlineStr">
+      <c r="E107" s="17" t="inlineStr">
         <is>
           <t>Important if specific ontology class not available</t>
         </is>
       </c>
-      <c r="F107" s="5" t="inlineStr">
+      <c r="F107" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
@@ -3529,24 +3563,24 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="5" t="inlineStr">
+      <c r="A109" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solvent B purity</t>
         </is>
       </c>
-      <c r="B109" s="5" t="n"/>
-      <c r="C109" s="5" t="inlineStr">
+      <c r="B109" s="17" t="n"/>
+      <c r="C109" s="17" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D109" s="5" t="inlineStr">
+      <c r="D109" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E109" s="5" t="n"/>
-      <c r="F109" s="5" t="inlineStr">
+      <c r="E109" s="17" t="n"/>
+      <c r="F109" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB-hasMeasuredProperty-Purity</t>
         </is>
@@ -3581,26 +3615,26 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="5" t="inlineStr">
+      <c r="A111" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solvent B volume fraction</t>
         </is>
       </c>
-      <c r="B111" s="5" t="n">
+      <c r="B111" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="C111" s="5" t="inlineStr">
+      <c r="C111" s="17" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D111" s="5" t="inlineStr">
+      <c r="D111" s="17" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E111" s="5" t="n"/>
-      <c r="F111" s="5" t="inlineStr">
+      <c r="E111" s="17" t="n"/>
+      <c r="F111" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
         </is>
@@ -3631,24 +3665,24 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="5" t="inlineStr">
+      <c r="A113" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solvent B manufacturer product ID</t>
         </is>
       </c>
-      <c r="B113" s="5" t="n"/>
-      <c r="C113" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D113" s="5" t="inlineStr">
+      <c r="B113" s="17" t="n"/>
+      <c r="C113" s="17" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D113" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E113" s="5" t="n"/>
-      <c r="F113" s="5" t="inlineStr">
+      <c r="E113" s="17" t="n"/>
+      <c r="F113" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolvent-hasConstituentB-schema:productID</t>
         </is>
@@ -3687,32 +3721,32 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="5" t="inlineStr">
+      <c r="A115" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solute A chemical name</t>
         </is>
       </c>
-      <c r="B115" s="5" t="inlineStr">
+      <c r="B115" s="17" t="inlineStr">
         <is>
           <t>KCrPDTA * 2 H2O (potassium [1,3-propylenediaminetetraacetato]chromate(III) dihydrate)</t>
         </is>
       </c>
-      <c r="C115" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D115" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E115" s="5" t="inlineStr">
+      <c r="C115" s="17" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D115" s="17" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E115" s="17" t="inlineStr">
         <is>
           <t>Important if specific ontology class not available</t>
         </is>
       </c>
-      <c r="F115" s="5" t="inlineStr">
+      <c r="F115" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
@@ -3751,26 +3785,26 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="5" t="inlineStr">
+      <c r="A117" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solute A purity</t>
         </is>
       </c>
-      <c r="B117" s="5" t="n">
+      <c r="B117" s="17" t="n">
         <v>99</v>
       </c>
-      <c r="C117" s="5" t="inlineStr">
+      <c r="C117" s="17" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D117" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E117" s="5" t="n"/>
-      <c r="F117" s="5" t="inlineStr">
+      <c r="D117" s="17" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E117" s="17" t="n"/>
+      <c r="F117" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-hasMeasuredProperty-Purity</t>
         </is>
@@ -3809,26 +3843,26 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="5" t="inlineStr">
+      <c r="A119" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Negative electrolyte solute A molarity </t>
         </is>
       </c>
-      <c r="B119" s="5" t="n">
+      <c r="B119" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C119" s="5" t="inlineStr">
+      <c r="C119" s="17" t="inlineStr">
         <is>
           <t>mol/L</t>
         </is>
       </c>
-      <c r="D119" s="5" t="inlineStr">
+      <c r="D119" s="17" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E119" s="5" t="n"/>
-      <c r="F119" s="5" t="inlineStr">
+      <c r="E119" s="17" t="n"/>
+      <c r="F119" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-hasMeasuredProperty-AmountConcentration</t>
         </is>
@@ -3863,28 +3897,28 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="inlineStr">
+      <c r="A121" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solute A manufacturer productD</t>
         </is>
       </c>
-      <c r="B121" s="5" t="inlineStr">
+      <c r="B121" s="17" t="inlineStr">
         <is>
           <t>KCrPDTA-Fall-25</t>
         </is>
       </c>
-      <c r="C121" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D121" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E121" s="5" t="n"/>
-      <c r="F121" s="5" t="inlineStr">
+      <c r="C121" s="17" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D121" s="17" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E121" s="17" t="n"/>
+      <c r="F121" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentA-schema:productID</t>
         </is>
@@ -3923,32 +3957,32 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="5" t="inlineStr">
+      <c r="A123" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solute B chemical name</t>
         </is>
       </c>
-      <c r="B123" s="5" t="inlineStr">
+      <c r="B123" s="17" t="inlineStr">
         <is>
           <t>H4PDTA (1,3-propylenediaminetetraacetic acid)</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D123" s="5" t="inlineStr">
+      <c r="C123" s="17" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D123" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E123" s="5" t="inlineStr">
+      <c r="E123" s="17" t="inlineStr">
         <is>
           <t>Important if specific ontology class not available</t>
         </is>
       </c>
-      <c r="F123" s="5" t="inlineStr">
+      <c r="F123" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
@@ -3987,26 +4021,26 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="5" t="inlineStr">
+      <c r="A125" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solute B purity</t>
         </is>
       </c>
-      <c r="B125" s="5" t="n">
+      <c r="B125" s="17" t="n">
         <v>99</v>
       </c>
-      <c r="C125" s="5" t="inlineStr">
+      <c r="C125" s="17" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D125" s="5" t="inlineStr">
+      <c r="D125" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E125" s="5" t="n"/>
-      <c r="F125" s="5" t="inlineStr">
+      <c r="E125" s="17" t="n"/>
+      <c r="F125" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-hasMeasuredProperty-Purity</t>
         </is>
@@ -4045,26 +4079,26 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="5" t="inlineStr">
+      <c r="A127" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solute B molarity</t>
         </is>
       </c>
-      <c r="B127" s="5" t="n">
+      <c r="B127" s="17" t="n">
         <v>0.1</v>
       </c>
-      <c r="C127" s="5" t="inlineStr">
+      <c r="C127" s="17" t="inlineStr">
         <is>
           <t>mol/L</t>
         </is>
       </c>
-      <c r="D127" s="5" t="inlineStr">
+      <c r="D127" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E127" s="5" t="n"/>
-      <c r="F127" s="5" t="inlineStr">
+      <c r="E127" s="17" t="n"/>
+      <c r="F127" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-hasMeasuredProperty-AmountConcentration</t>
         </is>
@@ -4099,26 +4133,26 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="5" t="inlineStr">
+      <c r="A129" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte solute B manufacturer product ID</t>
         </is>
       </c>
-      <c r="B129" s="5" t="n">
+      <c r="B129" s="17" t="n">
         <v>33267</v>
       </c>
-      <c r="C129" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D129" s="5" t="inlineStr">
+      <c r="C129" s="17" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D129" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E129" s="5" t="n"/>
-      <c r="F129" s="5" t="inlineStr">
+      <c r="E129" s="17" t="n"/>
+      <c r="F129" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasSolute-hasConstituentB-schema:productID</t>
         </is>
@@ -4151,26 +4185,26 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="inlineStr">
+      <c r="A131" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte volume flow rate</t>
         </is>
       </c>
-      <c r="B131" s="5" t="n">
+      <c r="B131" s="17" t="n">
         <v>60</v>
       </c>
-      <c r="C131" s="5" t="inlineStr">
+      <c r="C131" s="17" t="inlineStr">
         <is>
           <t>mL/min</t>
         </is>
       </c>
-      <c r="D131" s="5" t="inlineStr">
+      <c r="D131" s="17" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E131" s="5" t="n"/>
-      <c r="F131" s="5" t="inlineStr">
+      <c r="E131" s="17" t="n"/>
+      <c r="F131" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-VolumeFlowRate</t>
         </is>
@@ -4209,24 +4243,24 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="5" t="inlineStr">
+      <c r="A133" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte pressure</t>
         </is>
       </c>
-      <c r="B133" s="5" t="n"/>
-      <c r="C133" s="5" t="inlineStr">
+      <c r="B133" s="17" t="n"/>
+      <c r="C133" s="17" t="inlineStr">
         <is>
           <t>mbar</t>
         </is>
       </c>
-      <c r="D133" s="5" t="inlineStr">
+      <c r="D133" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E133" s="5" t="n"/>
-      <c r="F133" s="5" t="inlineStr">
+      <c r="E133" s="17" t="n"/>
+      <c r="F133" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-Pressure</t>
         </is>
@@ -4259,26 +4293,26 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="5" t="inlineStr">
+      <c r="A135" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte viscosity</t>
         </is>
       </c>
-      <c r="B135" s="5" t="n">
+      <c r="B135" s="17" t="n">
         <v>2.32</v>
       </c>
-      <c r="C135" s="5" t="inlineStr">
+      <c r="C135" s="17" t="inlineStr">
         <is>
           <t>mPa·s</t>
         </is>
       </c>
-      <c r="D135" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E135" s="5" t="n"/>
-      <c r="F135" s="5" t="inlineStr">
+      <c r="D135" s="17" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E135" s="17" t="n"/>
+      <c r="F135" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-DynamicViscosity</t>
         </is>
@@ -4311,26 +4345,26 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="5" t="inlineStr">
+      <c r="A137" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte density</t>
         </is>
       </c>
-      <c r="B137" s="5" t="n">
+      <c r="B137" s="17" t="n">
         <v>1.21</v>
       </c>
-      <c r="C137" s="5" t="inlineStr">
+      <c r="C137" s="17" t="inlineStr">
         <is>
           <t>g/cm3</t>
         </is>
       </c>
-      <c r="D137" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E137" s="5" t="n"/>
-      <c r="F137" s="5" t="inlineStr">
+      <c r="D137" s="17" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E137" s="17" t="n"/>
+      <c r="F137" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasMeasuredProperty-Density</t>
         </is>
@@ -4363,26 +4397,26 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="5" t="inlineStr">
+      <c r="A139" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte tank volume</t>
         </is>
       </c>
-      <c r="B139" s="5" t="n">
+      <c r="B139" s="17" t="n">
         <v>50</v>
       </c>
-      <c r="C139" s="5" t="inlineStr">
+      <c r="C139" s="17" t="inlineStr">
         <is>
           <t>mL</t>
         </is>
       </c>
-      <c r="D139" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E139" s="5" t="n"/>
-      <c r="F139" s="5" t="inlineStr">
+      <c r="D139" s="17" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E139" s="17" t="n"/>
+      <c r="F139" s="17" t="inlineStr">
         <is>
           <t>hasComponent-type|AnolyteTank-hasMeasuredProperty-Volume</t>
         </is>
@@ -4421,32 +4455,32 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="5" t="inlineStr">
+      <c r="A141" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte gas</t>
         </is>
       </c>
-      <c r="B141" s="5" t="inlineStr">
+      <c r="B141" s="17" t="inlineStr">
         <is>
           <t>Argon</t>
         </is>
       </c>
-      <c r="C141" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D141" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E141" s="5" t="inlineStr">
+      <c r="C141" s="17" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D141" s="17" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E141" s="17" t="inlineStr">
         <is>
           <t>e.g. Argon, Nitrogen, leave empty if none</t>
         </is>
       </c>
-      <c r="F141" s="5" t="inlineStr">
+      <c r="F141" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasBubbledGas</t>
         </is>
@@ -4479,42 +4513,42 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="5" t="inlineStr">
+      <c r="A143" s="17" t="inlineStr">
         <is>
           <t>Negative electrolyte gas pressure</t>
         </is>
       </c>
-      <c r="B143" s="5" t="n">
+      <c r="B143" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="C143" s="5" t="inlineStr">
+      <c r="C143" s="17" t="inlineStr">
         <is>
           <t>mbar</t>
         </is>
       </c>
-      <c r="D143" s="5" t="inlineStr">
+      <c r="D143" s="17" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E143" s="5" t="n"/>
-      <c r="F143" s="5" t="inlineStr">
+      <c r="E143" s="17" t="n"/>
+      <c r="F143" s="17" t="inlineStr">
         <is>
           <t>hasAnolyte-hasBubbledGas-hasMeasuredProperty-Pressure</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="inlineStr">
+      <c r="A144" s="18" t="inlineStr">
         <is>
           <t>Membrane</t>
         </is>
       </c>
-      <c r="B144" s="3" t="n"/>
-      <c r="C144" s="3" t="n"/>
-      <c r="D144" s="3" t="n"/>
-      <c r="E144" s="3" t="n"/>
-      <c r="F144" s="3" t="n"/>
+      <c r="B144" s="19" t="n"/>
+      <c r="C144" s="19" t="n"/>
+      <c r="D144" s="19" t="n"/>
+      <c r="E144" s="19" t="n"/>
+      <c r="F144" s="19" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -4549,28 +4583,28 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="5" t="inlineStr">
+      <c r="A146" s="20" t="inlineStr">
         <is>
           <t>Membrane A manufacturer</t>
         </is>
       </c>
-      <c r="B146" s="5" t="inlineStr">
+      <c r="B146" s="20" t="inlineStr">
         <is>
           <t>Fumatech</t>
         </is>
       </c>
-      <c r="C146" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D146" s="5" t="inlineStr">
+      <c r="C146" s="20" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D146" s="20" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E146" s="5" t="n"/>
-      <c r="F146" s="5" t="inlineStr">
+      <c r="E146" s="20" t="n"/>
+      <c r="F146" s="20" t="inlineStr">
         <is>
           <t>hasSeparator-schema:manufacturer</t>
         </is>
@@ -4605,32 +4639,32 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="5" t="inlineStr">
+      <c r="A148" s="20" t="inlineStr">
         <is>
           <t>Membrane material A class</t>
         </is>
       </c>
-      <c r="B148" s="5" t="inlineStr">
+      <c r="B148" s="20" t="inlineStr">
         <is>
           <t>PolyetherEtherKetone</t>
         </is>
       </c>
-      <c r="C148" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D148" s="5" t="inlineStr">
+      <c r="C148" s="20" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D148" s="20" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E148" s="5" t="inlineStr">
+      <c r="E148" s="20" t="inlineStr">
         <is>
           <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
-      <c r="F148" s="5" t="inlineStr">
+      <c r="F148" s="20" t="inlineStr">
         <is>
           <t>hasSeparator-hasConstituentA</t>
         </is>
@@ -4669,32 +4703,32 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="5" t="inlineStr">
+      <c r="A150" s="20" t="inlineStr">
         <is>
           <t>Membrane material A chemical formula</t>
         </is>
       </c>
-      <c r="B150" s="5" t="inlineStr">
+      <c r="B150" s="20" t="inlineStr">
         <is>
           <t>(C19H12O3)n</t>
         </is>
       </c>
-      <c r="C150" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D150" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E150" s="5" t="inlineStr">
+      <c r="C150" s="20" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D150" s="20" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E150" s="20" t="inlineStr">
         <is>
           <t>Important if specific ontology class not available</t>
         </is>
       </c>
-      <c r="F150" s="5" t="inlineStr">
+      <c r="F150" s="20" t="inlineStr">
         <is>
           <t>hasSeparator-hasConstituentA-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
@@ -4729,28 +4763,28 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="5" t="inlineStr">
+      <c r="A152" s="20" t="inlineStr">
         <is>
           <t>Membrane material B chemical name</t>
         </is>
       </c>
-      <c r="B152" s="5" t="n"/>
-      <c r="C152" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D152" s="5" t="inlineStr">
+      <c r="B152" s="20" t="n"/>
+      <c r="C152" s="20" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D152" s="20" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="E152" s="5" t="inlineStr">
+      <c r="E152" s="20" t="inlineStr">
         <is>
           <t>Important if specific ontology class not available</t>
         </is>
       </c>
-      <c r="F152" s="5" t="inlineStr">
+      <c r="F152" s="20" t="inlineStr">
         <is>
           <t>hasSeparator-hasConstituentB-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
@@ -4785,26 +4819,26 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="5" t="inlineStr">
+      <c r="A154" s="20" t="inlineStr">
         <is>
           <t>Membrane thickness</t>
         </is>
       </c>
-      <c r="B154" s="5" t="n">
+      <c r="B154" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="C154" s="5" t="inlineStr">
+      <c r="C154" s="20" t="inlineStr">
         <is>
           <t>um</t>
         </is>
       </c>
-      <c r="D154" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E154" s="5" t="n"/>
-      <c r="F154" s="5" t="inlineStr">
+      <c r="D154" s="20" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E154" s="20" t="n"/>
+      <c r="F154" s="20" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Thickness</t>
         </is>
@@ -4835,26 +4869,26 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="5" t="inlineStr">
+      <c r="A156" s="20" t="inlineStr">
         <is>
           <t>Membrane projected area</t>
         </is>
       </c>
-      <c r="B156" s="5" t="n">
+      <c r="B156" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C156" s="5" t="inlineStr">
+      <c r="C156" s="20" t="inlineStr">
         <is>
           <t>cm2</t>
         </is>
       </c>
-      <c r="D156" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E156" s="5" t="n"/>
-      <c r="F156" s="5" t="inlineStr">
+      <c r="D156" s="20" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E156" s="20" t="n"/>
+      <c r="F156" s="20" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Area</t>
         </is>
@@ -4893,48 +4927,48 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="5" t="inlineStr">
+      <c r="A158" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">Membrane pre-treatment </t>
         </is>
       </c>
-      <c r="B158" s="5" t="inlineStr">
+      <c r="B158" s="20" t="inlineStr">
         <is>
           <t>Untreated membrane</t>
         </is>
       </c>
-      <c r="C158" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D158" s="5" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E158" s="5" t="inlineStr">
+      <c r="C158" s="20" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D158" s="20" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E158" s="20" t="inlineStr">
         <is>
           <t>Describe membrane pre-treatment conditions (medium, duration, temperature)</t>
         </is>
       </c>
-      <c r="F158" s="5" t="inlineStr">
+      <c r="F158" s="20" t="inlineStr">
         <is>
           <t>hasSeparator-rdfs:comment</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="12" t="inlineStr">
+      <c r="A159" s="2" t="inlineStr">
         <is>
           <t>Cell assembly</t>
         </is>
       </c>
-      <c r="B159" s="13" t="n"/>
-      <c r="C159" s="13" t="n"/>
-      <c r="D159" s="13" t="n"/>
-      <c r="E159" s="13" t="n"/>
-      <c r="F159" s="13" t="n"/>
+      <c r="B159" s="3" t="n"/>
+      <c r="C159" s="3" t="n"/>
+      <c r="D159" s="3" t="n"/>
+      <c r="E159" s="3" t="n"/>
+      <c r="F159" s="3" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -4965,32 +4999,32 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="14" t="inlineStr">
+      <c r="A161" s="5" t="inlineStr">
         <is>
           <t>Cell case manufacturer</t>
         </is>
       </c>
-      <c r="B161" s="14" t="inlineStr">
+      <c r="B161" s="5" t="inlineStr">
         <is>
           <t>Fuel Cell Technologies</t>
         </is>
       </c>
-      <c r="C161" s="14" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D161" s="14" t="inlineStr">
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E161" s="14" t="inlineStr">
+      <c r="E161" s="5" t="inlineStr">
         <is>
           <t>Fuel Cell Technologies, Pinflow, etc.</t>
         </is>
       </c>
-      <c r="F161" s="14" t="inlineStr">
+      <c r="F161" s="5" t="inlineStr">
         <is>
           <t>hasCase-schema:manufacturer</t>
         </is>
@@ -5025,32 +5059,32 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="14" t="inlineStr">
+      <c r="A163" s="5" t="inlineStr">
         <is>
           <t>Flowfield material class</t>
         </is>
       </c>
-      <c r="B163" s="14" t="inlineStr">
+      <c r="B163" s="5" t="inlineStr">
         <is>
           <t>Graphite</t>
         </is>
       </c>
-      <c r="C163" s="14" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D163" s="14" t="inlineStr">
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E163" s="14" t="inlineStr">
+      <c r="E163" s="5" t="inlineStr">
         <is>
           <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
-      <c r="F163" s="14" t="inlineStr">
+      <c r="F163" s="5" t="inlineStr">
         <is>
           <t>hasComponent-type|FlowField</t>
         </is>
@@ -5089,32 +5123,32 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="14" t="inlineStr">
+      <c r="A165" s="5" t="inlineStr">
         <is>
           <t>Flowfield materail chemical formula</t>
         </is>
       </c>
-      <c r="B165" s="14" t="inlineStr">
+      <c r="B165" s="5" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C165" s="14" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D165" s="14" t="inlineStr">
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E165" s="14" t="inlineStr">
+      <c r="E165" s="5" t="inlineStr">
         <is>
           <t>Important if specific ontology class not available</t>
         </is>
       </c>
-      <c r="F165" s="14" t="inlineStr">
+      <c r="F165" s="5" t="inlineStr">
         <is>
           <t>hasComponent-type|FlowField-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
@@ -5149,28 +5183,28 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="14" t="inlineStr">
+      <c r="A167" s="5" t="inlineStr">
         <is>
           <t>Flowfield manufacturer</t>
         </is>
       </c>
-      <c r="B167" s="14" t="inlineStr">
+      <c r="B167" s="5" t="inlineStr">
         <is>
           <t>Fuel Cell Store</t>
         </is>
       </c>
-      <c r="C167" s="14" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D167" s="14" t="inlineStr">
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E167" s="14" t="n"/>
-      <c r="F167" s="14" t="inlineStr">
+      <c r="E167" s="5" t="n"/>
+      <c r="F167" s="5" t="inlineStr">
         <is>
           <t>hasComponent-type|FlowField-schema:manufacturer</t>
         </is>
@@ -5205,32 +5239,32 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="14" t="inlineStr">
+      <c r="A169" s="5" t="inlineStr">
         <is>
           <t>Gasket material class</t>
         </is>
       </c>
-      <c r="B169" s="14" t="inlineStr">
+      <c r="B169" s="5" t="inlineStr">
         <is>
           <t>PolymerCompound</t>
         </is>
       </c>
-      <c r="C169" s="14" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D169" s="14" t="inlineStr">
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E169" s="14" t="inlineStr">
+      <c r="E169" s="5" t="inlineStr">
         <is>
           <t>Ontology term, be as specific as possible</t>
         </is>
       </c>
-      <c r="F169" s="14" t="inlineStr">
+      <c r="F169" s="5" t="inlineStr">
         <is>
           <t>hasComponent-type|Gasket</t>
         </is>
@@ -5269,28 +5303,28 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="14" t="inlineStr">
+      <c r="A171" s="5" t="inlineStr">
         <is>
           <t>Gasket material chemical formula</t>
         </is>
       </c>
-      <c r="B171" s="14" t="n"/>
-      <c r="C171" s="14" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D171" s="14" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E171" s="14" t="inlineStr">
+      <c r="B171" s="5" t="n"/>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
         <is>
           <t>Important if specific ontology class not available</t>
         </is>
       </c>
-      <c r="F171" s="14" t="inlineStr">
+      <c r="F171" s="5" t="inlineStr">
         <is>
           <t>hasComponent-type|Gasket-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
@@ -5325,26 +5359,26 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="14" t="inlineStr">
+      <c r="A173" s="5" t="inlineStr">
         <is>
           <t>Gasket manufacturer product ID</t>
         </is>
       </c>
-      <c r="B173" s="14" t="n">
+      <c r="B173" s="5" t="n">
         <v>17965343</v>
       </c>
-      <c r="C173" s="14" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D173" s="14" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E173" s="14" t="n"/>
-      <c r="F173" s="14" t="inlineStr">
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D173" s="5" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="n"/>
+      <c r="F173" s="5" t="inlineStr">
         <is>
           <t>hasComponent-type|Gasket-schema:productID</t>
         </is>
@@ -5377,26 +5411,26 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="14" t="inlineStr">
+      <c r="A175" s="5" t="inlineStr">
         <is>
           <t>Torque upon assembly</t>
         </is>
       </c>
-      <c r="B175" s="14" t="n">
+      <c r="B175" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="C175" s="14" t="inlineStr">
+      <c r="C175" s="5" t="inlineStr">
         <is>
           <t>Nm</t>
         </is>
       </c>
-      <c r="D175" s="14" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E175" s="14" t="n"/>
-      <c r="F175" s="14" t="inlineStr">
+      <c r="D175" s="5" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E175" s="5" t="n"/>
+      <c r="F175" s="5" t="inlineStr">
         <is>
           <t>hasCase-hasMeasuredProperty-Torque</t>
         </is>
@@ -5435,32 +5469,32 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="14" t="inlineStr">
+      <c r="A177" s="5" t="inlineStr">
         <is>
           <t>Connection type</t>
         </is>
       </c>
-      <c r="B177" s="14" t="inlineStr">
+      <c r="B177" s="5" t="inlineStr">
         <is>
           <t>4-point</t>
         </is>
       </c>
-      <c r="C177" s="14" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
-      <c r="D177" s="14" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E177" s="14" t="inlineStr">
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>No Unit</t>
+        </is>
+      </c>
+      <c r="D177" s="5" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
         <is>
           <t>Describe if other mode, e.g. 2-point</t>
         </is>
       </c>
-      <c r="F177" s="14" t="inlineStr">
+      <c r="F177" s="5" t="inlineStr">
         <is>
           <t>hasComponent-type|Connector-rdfs:comment</t>
         </is>

</xml_diff>

<commit_message>
Update template and test data
</commit_message>
<xml_diff>
--- a/test/data/flowcell_excel_schema.xlsx
+++ b/test/data/flowcell_excel_schema.xlsx
@@ -2006,7 +2006,7 @@
       <c r="E52" s="14" t="n"/>
       <c r="F52" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolvent-hasConstituentA-hasMeasuredProperty-echem:Purity</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentA-hasMeasuredProperty-Purity</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       <c r="E60" s="14" t="n"/>
       <c r="F60" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolvent-hasConstituentB-hasMeasuredProperty-echem:Purity</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentB-hasMeasuredProperty-Purity</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       <c r="E68" s="14" t="n"/>
       <c r="F68" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolute-hasConstituentA-hasMeasuredProperty-echem:Purity</t>
+          <t>hasCatholyte-hasSolute-hasConstituentA-hasMeasuredProperty-Purity</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2686,7 @@
       <c r="E76" s="14" t="n"/>
       <c r="F76" s="14" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolute-hasConstituentB-hasMeasuredProperty-echem:Purity</t>
+          <t>hasCatholyte-hasSolute-hasConstituentB-hasMeasuredProperty-Purity</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
       <c r="E101" s="17" t="n"/>
       <c r="F101" s="17" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-hasConstituentA-hasMeasuredProperty-echem:Purity</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentA-hasMeasuredProperty-Purity</t>
         </is>
       </c>
     </row>
@@ -3582,7 +3582,7 @@
       <c r="E109" s="17" t="n"/>
       <c r="F109" s="17" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-hasConstituentB-hasMeasuredProperty-echem:Purity</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentB-hasMeasuredProperty-Purity</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3806,7 @@
       <c r="E117" s="17" t="n"/>
       <c r="F117" s="17" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-hasConstituentA-hasMeasuredProperty-echem:Purity</t>
+          <t>hasAnolyte-hasSolute-hasConstituentA-hasMeasuredProperty-Purity</t>
         </is>
       </c>
     </row>
@@ -4042,7 +4042,7 @@
       <c r="E125" s="17" t="n"/>
       <c r="F125" s="17" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-hasConstituentB-hasMeasuredProperty-echem:Purity</t>
+          <t>hasAnolyte-hasSolute-hasConstituentB-hasMeasuredProperty-Purity</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="F169" s="5" t="inlineStr">
         <is>
-          <t>hasComponent-type|echem:Gasket</t>
+          <t>hasComponent-type|Gasket</t>
         </is>
       </c>
     </row>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>hasComponent-type|echem:Gasket-hasDatumA-type|ChemicalName-hasStringValue</t>
+          <t>hasComponent-type|Gasket-hasDatumA-type|ChemicalName-hasStringValue</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="F171" s="5" t="inlineStr">
         <is>
-          <t>hasComponent-type|echem:Gasket-hasDatumB-type|ChemicalFormula-hasStringValue</t>
+          <t>hasComponent-type|Gasket-hasDatumB-type|ChemicalFormula-hasStringValue</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5354,7 @@
       <c r="E172" s="4" t="n"/>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>hasComponent-type|echem:Gasket-schema:manufacturer</t>
+          <t>hasComponent-type|Gasket-schema:manufacturer</t>
         </is>
       </c>
     </row>
@@ -5380,7 +5380,7 @@
       <c r="E173" s="5" t="n"/>
       <c r="F173" s="5" t="inlineStr">
         <is>
-          <t>hasComponent-type|echem:Gasket-schema:productID</t>
+          <t>hasComponent-type|Gasket-schema:productID</t>
         </is>
       </c>
     </row>

</xml_diff>